<commit_message>
added in file picker for selecting the location of the SA1 shapefile and calibrationRegions.csv, and with lowercase column names for origsa1 and destsa1 towards https://github.com/jibeproject/mito/issues/16
</commit_message>
<xml_diff>
--- a/dictionaries/VISTA_1220_data_dictionary_machine_readable.xlsx
+++ b/dictionaries/VISTA_1220_data_dictionary_machine_readable.xlsx
@@ -8447,9 +8447,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100481CAAAEC8DADD488E860CB2267F86FC" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8f98bb355169c9e617f40d43da358139">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="807c3283-625c-4b1c-9305-72cc1979a162" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="52358c6236a3fe3cc32594cf969eeac4" ns2:_="">
-    <xsd:import namespace="807c3283-625c-4b1c-9305-72cc1979a162"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C7E239D1F574DA47B0AD365A8221D720" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ea90b755d71099b3c5a1b2c34e23065f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="94c79151-e3b7-4a98-ac7f-99944fa0a67a" xmlns:ns3="ab102f35-6b42-4f6a-866b-1bf7020759a1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4e3ab1ac5f26c4059f5499449280014d" ns2:_="" ns3:_="">
+    <xsd:import namespace="94c79151-e3b7-4a98-ac7f-99944fa0a67a"/>
+    <xsd:import namespace="ab102f35-6b42-4f6a-866b-1bf7020759a1"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -8458,8 +8459,17 @@
               <xsd:all>
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -8467,7 +8477,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="807c3283-625c-4b1c-9305-72cc1979a162" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="94c79151-e3b7-4a98-ac7f-99944fa0a67a" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -8480,14 +8490,89 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="10" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="12" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="c921d02d-b337-4ce5-bd1c-22d9132a6b17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="14" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="17" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ab102f35-6b42-4f6a-866b-1bf7020759a1" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="13" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{d3a442e0-bfe2-4df2-a0d1-057535b81225}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ab102f35-6b42-4f6a-866b-1bf7020759a1">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="20" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="21" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -8599,22 +8684,19 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ab102f35-6b42-4f6a-866b-1bf7020759a1" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="94c79151-e3b7-4a98-ac7f-99944fa0a67a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4D1FB37-B5C9-4E67-96A3-9E18CFE05286}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="807c3283-625c-4b1c-9305-72cc1979a162"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97A230A6-99BC-48CE-8C04-6299A24FE2DF}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8623,4 +8705,8 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FC1DCD7-8B43-4ECE-9B59-F04A6549A4BA}"/>
 </file>
</xml_diff>